<commit_message>
chore(public): update excel templates
Update the binary Excel templates for Sibuhar and Simpanan to reflect recent changes in data structure or requirements.
</commit_message>
<xml_diff>
--- a/public/template_sibuhar.xlsx
+++ b/public/template_sibuhar.xlsx
@@ -418,7 +418,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>001</v>
+        <v>1</v>
       </c>
       <c r="B2" t="str">
         <v>Contoh Anggota 1</v>
@@ -435,7 +435,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>002</v>
+        <v>2</v>
       </c>
       <c r="B3" t="str">
         <v>Contoh Anggota 2</v>

</xml_diff>

<commit_message>
chore(public): update sibuhar excel template
</commit_message>
<xml_diff>
--- a/public/template_sibuhar.xlsx
+++ b/public/template_sibuhar.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -450,9 +450,26 @@
         <v>150000</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Contoh Anggota 3</v>
+      </c>
+      <c r="C4" t="str">
+        <v>17-01-2024</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Penarikan</v>
+      </c>
+      <c r="E4">
+        <v>50000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>